<commit_message>
Updated CV matching logic using semantic similarity
</commit_message>
<xml_diff>
--- a/Performance_Productivity/Prediction_Result/prediction_results.xlsx
+++ b/Performance_Productivity/Prediction_Result/prediction_results.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O16"/>
+  <dimension ref="A1:P34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -482,25 +482,30 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Predicted_Productivity_Percentage</t>
+          <t>FeedBack</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
+          <t>Predicted_Productivity</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
           <t>Productivity_Class</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Predicted_Productivity_Risk</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Recommendations</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Output_Summary</t>
         </is>
@@ -509,7 +514,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>EMP001</t>
+          <t>ID001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -544,33 +549,36 @@
         <v>30</v>
       </c>
       <c r="K2" t="n">
-        <v>96.48999786376953</v>
-      </c>
-      <c r="L2" t="inlineStr">
+        <v>92.45</v>
+      </c>
+      <c r="L2" t="n">
+        <v>98.52</v>
+      </c>
+      <c r="M2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
       <c r="N2" t="inlineStr">
         <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
           <t>Monitor workload</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>Employee productivity is predicted to be 96.49%. Productivity class: High. Risk level: Low. Recommended action: Monitor workload.</t>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Employee productivity percentage is predicted to be 98.52%. Productivity class: High. Risk level: Low. Recommended action: Monitor workload.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>EMP002</t>
+          <t>ID002</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -605,33 +613,36 @@
         <v>12</v>
       </c>
       <c r="K3" t="n">
-        <v>53.2599983215332</v>
-      </c>
-      <c r="L3" t="inlineStr">
+        <v>41.8</v>
+      </c>
+      <c r="L3" t="n">
+        <v>32.71</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>Reduce overtime; Increase training; Monitor workload; Improve task completion</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>Employee productivity is predicted to be 53.26%. Productivity class: Medium. Risk level: Medium. Recommended action: Reduce overtime; Increase training; Monitor workload; Improve task completion.</t>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Employee productivity percentage is predicted to be 32.71%. Productivity class: Low. Risk level: Medium. Recommended action: Reduce overtime; Increase training; Monitor workload; Improve task completion.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>EMP003</t>
+          <t>ID003</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -666,33 +677,36 @@
         <v>8</v>
       </c>
       <c r="K4" t="n">
-        <v>21.98999977111816</v>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
+        <v>22.35</v>
+      </c>
+      <c r="L4" t="n">
+        <v>9.300000000000001</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>Improve attendance; Reduce overtime; Increase training; Monitor workload; Improve task completion</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>Employee productivity is predicted to be 21.99%. Productivity class: Low. Risk level: High. Recommended action: Improve attendance; Reduce overtime; Increase training; Monitor workload; Improve task completion.</t>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Employee productivity percentage is predicted to be 9.30%. Productivity class: Low. Risk level: High. Recommended action: Improve attendance; Reduce overtime; Increase training; Monitor workload; Improve task completion.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>EMP004</t>
+          <t>ID004</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -727,33 +741,36 @@
         <v>22</v>
       </c>
       <c r="K5" t="n">
-        <v>96.31999969482422</v>
-      </c>
-      <c r="L5" t="inlineStr">
+        <v>78.59999999999999</v>
+      </c>
+      <c r="L5" t="n">
+        <v>96.44</v>
+      </c>
+      <c r="M5" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
       <c r="N5" t="inlineStr">
         <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
           <t>Monitor workload</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>Employee productivity is predicted to be 96.32%. Productivity class: High. Risk level: Low. Recommended action: Monitor workload.</t>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Employee productivity percentage is predicted to be 96.44%. Productivity class: High. Risk level: Low. Recommended action: Monitor workload.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>EMP005</t>
+          <t>ID005</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -788,12 +805,10 @@
         <v>15</v>
       </c>
       <c r="K6" t="n">
-        <v>79.27999877929688</v>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
+        <v>61.25</v>
+      </c>
+      <c r="L6" t="n">
+        <v>56.7</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
@@ -802,19 +817,24 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
           <t>Reduce overtime; Monitor workload</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>Employee productivity is predicted to be 79.28%. Productivity class: High. Risk level: Medium. Recommended action: Reduce overtime; Monitor workload.</t>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Employee productivity percentage is predicted to be 56.70%. Productivity class: Medium. Risk level: Medium. Recommended action: Reduce overtime; Monitor workload.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>EMP006</t>
+          <t>ID006</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -849,33 +869,36 @@
         <v>28</v>
       </c>
       <c r="K7" t="n">
-        <v>96.58000183105469</v>
-      </c>
-      <c r="L7" t="inlineStr">
+        <v>94.09999999999999</v>
+      </c>
+      <c r="L7" t="n">
+        <v>98.5</v>
+      </c>
+      <c r="M7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
       <c r="N7" t="inlineStr">
         <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
           <t>Monitor workload</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>Employee productivity is predicted to be 96.58%. Productivity class: High. Risk level: Low. Recommended action: Monitor workload.</t>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Employee productivity percentage is predicted to be 98.50%. Productivity class: High. Risk level: Low. Recommended action: Monitor workload.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>EMP007</t>
+          <t>ID007</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -910,33 +933,36 @@
         <v>10</v>
       </c>
       <c r="K8" t="n">
-        <v>36.22000122070312</v>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
+        <v>36.9</v>
+      </c>
+      <c r="L8" t="n">
+        <v>16.33</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>Improve attendance; Reduce overtime; Increase training; Monitor workload; Improve task completion</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>Employee productivity is predicted to be 36.22%. Productivity class: Low. Risk level: High. Recommended action: Improve attendance; Reduce overtime; Increase training; Monitor workload; Improve task completion.</t>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Employee productivity percentage is predicted to be 16.33%. Productivity class: Low. Risk level: High. Recommended action: Improve attendance; Reduce overtime; Increase training; Monitor workload; Improve task completion.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>EMP008</t>
+          <t>ID008</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -971,33 +997,36 @@
         <v>20</v>
       </c>
       <c r="K9" t="n">
-        <v>96.41000366210938</v>
-      </c>
-      <c r="L9" t="inlineStr">
+        <v>84.75</v>
+      </c>
+      <c r="L9" t="n">
+        <v>96.56999999999999</v>
+      </c>
+      <c r="M9" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
       <c r="N9" t="inlineStr">
         <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
           <t>Monitor workload</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>Employee productivity is predicted to be 96.41%. Productivity class: High. Risk level: Low. Recommended action: Monitor workload.</t>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Employee productivity percentage is predicted to be 96.57%. Productivity class: High. Risk level: Low. Recommended action: Monitor workload.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>EMP009</t>
+          <t>ID009</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1032,33 +1061,36 @@
         <v>14</v>
       </c>
       <c r="K10" t="n">
-        <v>72.37000274658203</v>
-      </c>
-      <c r="L10" t="inlineStr">
+        <v>58.45</v>
+      </c>
+      <c r="L10" t="n">
+        <v>51.91</v>
+      </c>
+      <c r="M10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
+      <c r="O10" t="inlineStr">
         <is>
           <t>Reduce overtime; Increase training; Monitor workload</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>Employee productivity is predicted to be 72.37%. Productivity class: Medium. Risk level: Medium. Recommended action: Reduce overtime; Increase training; Monitor workload.</t>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Employee productivity percentage is predicted to be 51.91%. Productivity class: Medium. Risk level: Medium. Recommended action: Reduce overtime; Increase training; Monitor workload.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>EMP010</t>
+          <t>ID010</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1093,33 +1125,36 @@
         <v>6</v>
       </c>
       <c r="K11" t="n">
-        <v>19.70999908447266</v>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
+        <v>15.8</v>
+      </c>
+      <c r="L11" t="n">
+        <v>10.16</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
+      <c r="O11" t="inlineStr">
         <is>
           <t>Improve attendance; Reduce overtime; Increase training; Monitor workload; Improve task completion</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>Employee productivity is predicted to be 19.71%. Productivity class: Low. Risk level: High. Recommended action: Improve attendance; Reduce overtime; Increase training; Monitor workload; Improve task completion.</t>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Employee productivity percentage is predicted to be 10.16%. Productivity class: Low. Risk level: High. Recommended action: Improve attendance; Reduce overtime; Increase training; Monitor workload; Improve task completion.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>EMP011</t>
+          <t>ID011</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1154,33 +1189,36 @@
         <v>35</v>
       </c>
       <c r="K12" t="n">
-        <v>96.59999847412109</v>
-      </c>
-      <c r="L12" t="inlineStr">
+        <v>97.2</v>
+      </c>
+      <c r="L12" t="n">
+        <v>99.05</v>
+      </c>
+      <c r="M12" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
       <c r="N12" t="inlineStr">
         <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
           <t>Monitor workload</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>Employee productivity is predicted to be 96.60%. Productivity class: High. Risk level: Low. Recommended action: Monitor workload.</t>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>Employee productivity percentage is predicted to be 99.05%. Productivity class: High. Risk level: Low. Recommended action: Monitor workload.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>EMP012</t>
+          <t>ID012</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1215,33 +1253,36 @@
         <v>18</v>
       </c>
       <c r="K13" t="n">
-        <v>87.22000122070312</v>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
+        <v>69.34999999999999</v>
+      </c>
+      <c r="L13" t="n">
+        <v>74.23999999999999</v>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
           <t>Maintain current performance</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>Employee productivity is predicted to be 87.22%. Productivity class: High. Risk level: Low. Recommended action: Maintain current performance.</t>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>Employee productivity percentage is predicted to be 74.24%. Productivity class: Medium. Risk level: Low. Recommended action: Maintain current performance.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>EMP013</t>
+          <t>ID013</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1276,33 +1317,36 @@
         <v>25</v>
       </c>
       <c r="K14" t="n">
-        <v>96.33000183105469</v>
-      </c>
-      <c r="L14" t="inlineStr">
+        <v>88.40000000000001</v>
+      </c>
+      <c r="L14" t="n">
+        <v>98.42</v>
+      </c>
+      <c r="M14" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
       <c r="N14" t="inlineStr">
         <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
           <t>Monitor workload</t>
         </is>
       </c>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>Employee productivity is predicted to be 96.33%. Productivity class: High. Risk level: Low. Recommended action: Monitor workload.</t>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>Employee productivity percentage is predicted to be 98.42%. Productivity class: High. Risk level: Low. Recommended action: Monitor workload.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>EMP014</t>
+          <t>ID014</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1337,33 +1381,36 @@
         <v>9</v>
       </c>
       <c r="K15" t="n">
-        <v>27.06999969482422</v>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
+        <v>31.65</v>
+      </c>
+      <c r="L15" t="n">
+        <v>12.53</v>
       </c>
       <c r="M15" t="inlineStr">
         <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr">
+      <c r="O15" t="inlineStr">
         <is>
           <t>Improve attendance; Reduce overtime; Increase training; Monitor workload; Improve task completion</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>Employee productivity is predicted to be 27.07%. Productivity class: Low. Risk level: High. Recommended action: Improve attendance; Reduce overtime; Increase training; Monitor workload; Improve task completion.</t>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>Employee productivity percentage is predicted to be 12.53%. Productivity class: Low. Risk level: High. Recommended action: Improve attendance; Reduce overtime; Increase training; Monitor workload; Improve task completion.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>EMP015</t>
+          <t>ID015</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1398,26 +1445,1181 @@
         <v>16</v>
       </c>
       <c r="K16" t="n">
-        <v>83.55000305175781</v>
-      </c>
-      <c r="L16" t="inlineStr">
+        <v>54.75</v>
+      </c>
+      <c r="L16" t="n">
+        <v>61.08</v>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>Maintain current performance</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>Employee productivity percentage is predicted to be 61.08%. Productivity class: Medium. Risk level: Low. Recommended action: Maintain current performance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>ID016</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Business Analyst</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>52</v>
+      </c>
+      <c r="E17" t="n">
+        <v>28</v>
+      </c>
+      <c r="F17" t="n">
+        <v>5</v>
+      </c>
+      <c r="G17" t="n">
+        <v>5</v>
+      </c>
+      <c r="H17" t="n">
+        <v>22</v>
+      </c>
+      <c r="I17" t="n">
+        <v>14</v>
+      </c>
+      <c r="J17" t="n">
+        <v>32</v>
+      </c>
+      <c r="K17" t="n">
+        <v>96.84999999999999</v>
+      </c>
+      <c r="L17" t="n">
+        <v>98.94</v>
+      </c>
+      <c r="M17" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>Maintain current performance</t>
-        </is>
-      </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>Employee productivity is predicted to be 83.55%. Productivity class: High. Risk level: Low. Recommended action: Maintain current performance.</t>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>Monitor workload</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>Employee productivity percentage is predicted to be 98.94%. Productivity class: High. Risk level: Low. Recommended action: Monitor workload.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>ID017</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Solution Architect</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>48</v>
+      </c>
+      <c r="E18" t="n">
+        <v>23</v>
+      </c>
+      <c r="F18" t="n">
+        <v>5</v>
+      </c>
+      <c r="G18" t="n">
+        <v>5</v>
+      </c>
+      <c r="H18" t="n">
+        <v>18</v>
+      </c>
+      <c r="I18" t="n">
+        <v>12</v>
+      </c>
+      <c r="J18" t="n">
+        <v>30</v>
+      </c>
+      <c r="K18" t="n">
+        <v>91.59999999999999</v>
+      </c>
+      <c r="L18" t="n">
+        <v>98.7</v>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>Monitor workload</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>Employee productivity percentage is predicted to be 98.70%. Productivity class: High. Risk level: Low. Recommended action: Monitor workload.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>ID018</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>System Analyst</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>29</v>
+      </c>
+      <c r="E19" t="n">
+        <v>5</v>
+      </c>
+      <c r="F19" t="n">
+        <v>3</v>
+      </c>
+      <c r="G19" t="n">
+        <v>3</v>
+      </c>
+      <c r="H19" t="n">
+        <v>7</v>
+      </c>
+      <c r="I19" t="n">
+        <v>28</v>
+      </c>
+      <c r="J19" t="n">
+        <v>12</v>
+      </c>
+      <c r="K19" t="n">
+        <v>63.9</v>
+      </c>
+      <c r="L19" t="n">
+        <v>50.47</v>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>Reduce overtime; Increase training; Monitor workload</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>Employee productivity percentage is predicted to be 50.47%. Productivity class: Medium. Risk level: Medium. Recommended action: Reduce overtime; Increase training; Monitor workload.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>ID019</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Trainee</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>UX Researcher</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>24</v>
+      </c>
+      <c r="E20" t="n">
+        <v>2</v>
+      </c>
+      <c r="F20" t="n">
+        <v>2</v>
+      </c>
+      <c r="G20" t="n">
+        <v>2</v>
+      </c>
+      <c r="H20" t="n">
+        <v>3</v>
+      </c>
+      <c r="I20" t="n">
+        <v>35</v>
+      </c>
+      <c r="J20" t="n">
+        <v>10</v>
+      </c>
+      <c r="K20" t="n">
+        <v>38.25</v>
+      </c>
+      <c r="L20" t="n">
+        <v>14.26</v>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>Improve attendance; Reduce overtime; Increase training; Monitor workload; Improve task completion</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>Employee productivity percentage is predicted to be 14.26%. Productivity class: Low. Risk level: High. Recommended action: Improve attendance; Reduce overtime; Increase training; Monitor workload; Improve task completion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>ID020</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Cloud Engineer</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>41</v>
+      </c>
+      <c r="E21" t="n">
+        <v>17</v>
+      </c>
+      <c r="F21" t="n">
+        <v>4</v>
+      </c>
+      <c r="G21" t="n">
+        <v>4</v>
+      </c>
+      <c r="H21" t="n">
+        <v>14</v>
+      </c>
+      <c r="I21" t="n">
+        <v>20</v>
+      </c>
+      <c r="J21" t="n">
+        <v>25</v>
+      </c>
+      <c r="K21" t="n">
+        <v>82.55</v>
+      </c>
+      <c r="L21" t="n">
+        <v>96.59999999999999</v>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>Monitor workload</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>Employee productivity percentage is predicted to be 96.60%. Productivity class: High. Risk level: Low. Recommended action: Monitor workload.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>ID021</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>QA Engineer</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>27</v>
+      </c>
+      <c r="E22" t="n">
+        <v>4</v>
+      </c>
+      <c r="F22" t="n">
+        <v>3</v>
+      </c>
+      <c r="G22" t="n">
+        <v>3</v>
+      </c>
+      <c r="H22" t="n">
+        <v>6</v>
+      </c>
+      <c r="I22" t="n">
+        <v>30</v>
+      </c>
+      <c r="J22" t="n">
+        <v>14</v>
+      </c>
+      <c r="K22" t="n">
+        <v>57.3</v>
+      </c>
+      <c r="L22" t="n">
+        <v>46.38</v>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>Reduce overtime; Increase training; Monitor workload</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>Employee productivity percentage is predicted to be 46.38%. Productivity class: Low. Risk level: Medium. Recommended action: Reduce overtime; Increase training; Monitor workload.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>ID022</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Data Engineer</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>45</v>
+      </c>
+      <c r="E23" t="n">
+        <v>20</v>
+      </c>
+      <c r="F23" t="n">
+        <v>5</v>
+      </c>
+      <c r="G23" t="n">
+        <v>5</v>
+      </c>
+      <c r="H23" t="n">
+        <v>16</v>
+      </c>
+      <c r="I23" t="n">
+        <v>18</v>
+      </c>
+      <c r="J23" t="n">
+        <v>28</v>
+      </c>
+      <c r="K23" t="n">
+        <v>93.75</v>
+      </c>
+      <c r="L23" t="n">
+        <v>98.55</v>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>Monitor workload</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>Employee productivity percentage is predicted to be 98.55%. Productivity class: High. Risk level: Low. Recommended action: Monitor workload.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>ID023</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>UX Engineer</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>43</v>
+      </c>
+      <c r="E24" t="n">
+        <v>20</v>
+      </c>
+      <c r="F24" t="n">
+        <v>3</v>
+      </c>
+      <c r="G24" t="n">
+        <v>2</v>
+      </c>
+      <c r="H24" t="n">
+        <v>12</v>
+      </c>
+      <c r="I24" t="n">
+        <v>24</v>
+      </c>
+      <c r="J24" t="n">
+        <v>21</v>
+      </c>
+      <c r="K24" t="n">
+        <v>72.65000000000001</v>
+      </c>
+      <c r="L24" t="n">
+        <v>60.02</v>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>Improve attendance; Monitor workload</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>Employee productivity percentage is predicted to be 60.02%. Productivity class: Medium. Risk level: Low. Recommended action: Improve attendance; Monitor workload.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>ID024</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>UX Engineer</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>43</v>
+      </c>
+      <c r="E25" t="n">
+        <v>12</v>
+      </c>
+      <c r="F25" t="n">
+        <v>3</v>
+      </c>
+      <c r="G25" t="n">
+        <v>2</v>
+      </c>
+      <c r="H25" t="n">
+        <v>12</v>
+      </c>
+      <c r="I25" t="n">
+        <v>24</v>
+      </c>
+      <c r="J25" t="n">
+        <v>21</v>
+      </c>
+      <c r="K25" t="n">
+        <v>66.40000000000001</v>
+      </c>
+      <c r="L25" t="n">
+        <v>59.41</v>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>Improve attendance; Monitor workload</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>Employee productivity percentage is predicted to be 59.41%. Productivity class: Medium. Risk level: Low. Recommended action: Improve attendance; Monitor workload.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>ID025</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Trainee</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Software Engineer</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>23</v>
+      </c>
+      <c r="E26" t="n">
+        <v>2</v>
+      </c>
+      <c r="F26" t="n">
+        <v>4</v>
+      </c>
+      <c r="G26" t="n">
+        <v>2</v>
+      </c>
+      <c r="H26" t="n">
+        <v>12</v>
+      </c>
+      <c r="I26" t="n">
+        <v>24</v>
+      </c>
+      <c r="J26" t="n">
+        <v>21</v>
+      </c>
+      <c r="K26" t="n">
+        <v>49.55</v>
+      </c>
+      <c r="L26" t="n">
+        <v>56.41</v>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>Improve attendance; Monitor workload</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>Employee productivity percentage is predicted to be 56.41%. Productivity class: Medium. Risk level: Medium. Recommended action: Improve attendance; Monitor workload.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>ID026</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Trainee</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Software Engineer</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>23</v>
+      </c>
+      <c r="E27" t="n">
+        <v>1</v>
+      </c>
+      <c r="F27" t="n">
+        <v>3</v>
+      </c>
+      <c r="G27" t="n">
+        <v>4</v>
+      </c>
+      <c r="H27" t="n">
+        <v>10</v>
+      </c>
+      <c r="I27" t="n">
+        <v>23</v>
+      </c>
+      <c r="J27" t="n">
+        <v>20</v>
+      </c>
+      <c r="K27" t="n">
+        <v>52.8</v>
+      </c>
+      <c r="L27" t="n">
+        <v>72.01000000000001</v>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>Monitor workload</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>Employee productivity percentage is predicted to be 72.01%. Productivity class: Medium. Risk level: Low. Recommended action: Monitor workload.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>ID027</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Cloud Engineer</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>41</v>
+      </c>
+      <c r="E28" t="n">
+        <v>17</v>
+      </c>
+      <c r="F28" t="n">
+        <v>4</v>
+      </c>
+      <c r="G28" t="n">
+        <v>4</v>
+      </c>
+      <c r="H28" t="n">
+        <v>14</v>
+      </c>
+      <c r="I28" t="n">
+        <v>20</v>
+      </c>
+      <c r="J28" t="n">
+        <v>25</v>
+      </c>
+      <c r="K28" t="n">
+        <v>86.3</v>
+      </c>
+      <c r="L28" t="n">
+        <v>96.59999999999999</v>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>Monitor workload</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>Employee productivity percentage is predicted to be 96.60%. Productivity class: High. Risk level: Low. Recommended action: Monitor workload.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>ID028</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Cloud Engineer</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>41</v>
+      </c>
+      <c r="E29" t="n">
+        <v>8</v>
+      </c>
+      <c r="F29" t="n">
+        <v>2</v>
+      </c>
+      <c r="G29" t="n">
+        <v>2</v>
+      </c>
+      <c r="H29" t="n">
+        <v>5</v>
+      </c>
+      <c r="I29" t="n">
+        <v>10</v>
+      </c>
+      <c r="J29" t="n">
+        <v>15</v>
+      </c>
+      <c r="K29" t="n">
+        <v>59.7</v>
+      </c>
+      <c r="L29" t="n">
+        <v>40.21</v>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>Improve attendance; Monitor workload; Improve task completion</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>Employee productivity percentage is predicted to be 40.21%. Productivity class: Low. Risk level: Medium. Recommended action: Improve attendance; Monitor workload; Improve task completion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>ID100</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>UI Designer</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>32</v>
+      </c>
+      <c r="E30" t="n">
+        <v>10</v>
+      </c>
+      <c r="F30" t="n">
+        <v>2</v>
+      </c>
+      <c r="G30" t="n">
+        <v>3</v>
+      </c>
+      <c r="H30" t="n">
+        <v>16</v>
+      </c>
+      <c r="I30" t="n">
+        <v>48</v>
+      </c>
+      <c r="J30" t="n">
+        <v>2</v>
+      </c>
+      <c r="K30" t="n">
+        <v>78.59999999999999</v>
+      </c>
+      <c r="L30" t="n">
+        <v>34.34</v>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>Reduce overtime; Increase training; Monitor workload; Improve task completion</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>Employee productivity percentage is predicted to be 34.34%. Productivity class: Low. Risk level: Medium. Recommended action: Reduce overtime; Increase training; Monitor workload; Improve task completion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>ID101</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>UI Designer</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>42</v>
+      </c>
+      <c r="E31" t="n">
+        <v>8</v>
+      </c>
+      <c r="F31" t="n">
+        <v>4</v>
+      </c>
+      <c r="G31" t="n">
+        <v>3</v>
+      </c>
+      <c r="H31" t="n">
+        <v>13</v>
+      </c>
+      <c r="I31" t="n">
+        <v>42</v>
+      </c>
+      <c r="J31" t="n">
+        <v>6</v>
+      </c>
+      <c r="K31" t="n">
+        <v>74.5</v>
+      </c>
+      <c r="L31" t="n">
+        <v>66.83</v>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>Reduce overtime; Increase training; Monitor workload</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>Employee productivity percentage is predicted to be 66.83%. Productivity class: Medium. Risk level: Low. Recommended action: Reduce overtime; Increase training; Monitor workload.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>ID102</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Trainee</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>UI Designer</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>26</v>
+      </c>
+      <c r="E32" t="n">
+        <v>3</v>
+      </c>
+      <c r="F32" t="n">
+        <v>4</v>
+      </c>
+      <c r="G32" t="n">
+        <v>4</v>
+      </c>
+      <c r="H32" t="n">
+        <v>7</v>
+      </c>
+      <c r="I32" t="n">
+        <v>10</v>
+      </c>
+      <c r="J32" t="n">
+        <v>10</v>
+      </c>
+      <c r="K32" t="n">
+        <v>84.5</v>
+      </c>
+      <c r="L32" t="n">
+        <v>89.26000000000001</v>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>Increase training</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>Employee productivity percentage is predicted to be 89.26%. Productivity class: High. Risk level: Low. Recommended action: Increase training.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>ID201</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Software Engineer</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>32</v>
+      </c>
+      <c r="E33" t="n">
+        <v>10</v>
+      </c>
+      <c r="F33" t="n">
+        <v>4</v>
+      </c>
+      <c r="G33" t="n">
+        <v>3</v>
+      </c>
+      <c r="H33" t="n">
+        <v>16</v>
+      </c>
+      <c r="I33" t="n">
+        <v>48</v>
+      </c>
+      <c r="J33" t="n">
+        <v>10</v>
+      </c>
+      <c r="K33" t="n">
+        <v>78.59999999999999</v>
+      </c>
+      <c r="L33" t="n">
+        <v>71.26000000000001</v>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>Reduce overtime; Increase training; Monitor workload</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>Employee productivity percentage is predicted to be 71.26%. Productivity class: Medium. Risk level: Low. Recommended action: Reduce overtime; Increase training; Monitor workload.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>ID202</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Software Engineer</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>42</v>
+      </c>
+      <c r="E34" t="n">
+        <v>8</v>
+      </c>
+      <c r="F34" t="n">
+        <v>4</v>
+      </c>
+      <c r="G34" t="n">
+        <v>3</v>
+      </c>
+      <c r="H34" t="n">
+        <v>13</v>
+      </c>
+      <c r="I34" t="n">
+        <v>42</v>
+      </c>
+      <c r="J34" t="n">
+        <v>6</v>
+      </c>
+      <c r="K34" t="n">
+        <v>74.5</v>
+      </c>
+      <c r="L34" t="n">
+        <v>66.83</v>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>Reduce overtime; Increase training; Monitor workload</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>Employee productivity percentage is predicted to be 66.83%. Productivity class: Medium. Risk level: Low. Recommended action: Reduce overtime; Increase training; Monitor workload.</t>
         </is>
       </c>
     </row>
@@ -1454,7 +2656,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>15</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3">
@@ -1464,7 +2666,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>70.62999725341797</v>
+        <v>64.53</v>
       </c>
     </row>
     <row r="4">
@@ -1474,7 +2676,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>19.70999908447266</v>
+        <v>9.300000000000001</v>
       </c>
     </row>
     <row r="5">
@@ -1484,7 +2686,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>96.59999847412109</v>
+        <v>99.05</v>
       </c>
     </row>
     <row r="6">
@@ -1494,7 +2696,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7">
@@ -1504,7 +2706,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8">
@@ -1514,7 +2716,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9">
@@ -1524,7 +2726,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10">
@@ -1534,7 +2736,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11">
@@ -1544,7 +2746,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>